<commit_message>
DOC 21b: Banco de Hooks v3.2 alineado al Spine post-contraste
36 hooks que abren por el terror del diagnostico de higado graso + revertir sin
cirugia (deroga el frame v3 de hinchazon estetica). Cada hook con ID de cita real,
inferencia, cluster, hipotesis que testea y prioridad de testeo. 3 lentes: nucleo
diagnostico / seguridad-prueba-mecanismo / cabeza de playa hinchazon (a validar).
+ pestana 'Hooks v3.2' en el Excel consolidado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSOLIDADO — Research Hígado MX.xlsx
+++ b/CONSOLIDADO — Research Hígado MX.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hooks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competencia" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avatares (Tier)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deseos (PI Tier)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecanismos (UMP-UMS-USP)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oportunidades y Mejoras" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hooks v3.2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competencia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avatares (Tier)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deseos (PI Tier)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecanismos (UMP-UMS-USP)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oportunidades y Mejoras" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +73,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="15"/>
     </font>
   </fonts>
   <fills count="8">
@@ -138,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,6 +189,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2040,6 +2056,1787 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>BANCO DE HOOKS v3.2 (alineado al Spine post-contraste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>📄 Ver documento: DOC 21b — Banco de Hooks v3.2 (supera al DOC 21 v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Lente</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Hook</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Conciencia</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Sub-avatar</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>ID origen</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Hipótesis que testea</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Formato</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Ayer lloré y lloré: a mi hija de 25 le detectaron hígado graso. Dije: Dios mío, ¿ahora qué hago?</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Inconsciente</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Terror del diagnóstico / madre por la hija</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>EV20ee996cc059</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Abrir por el diagnóstico de un hijo (no propio) engancha más fuerte el terror que abrir por el diagnóstico propio.</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>El 30 de mayo enterré a mi sobrina de 33. Buena, llena de vida. Se la llevó el hígado graso y la diabetes.</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Inconsciente</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Miedo mortal / vi morir a alguien</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>EV8c9dc6159962</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>El testimonio de una muerte cercana joven convierte el hígado graso de molestia a amenaza mortal más que una estadística.</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Me detectaron hígado graso y cálculos en la vesícula. En mi desesperación probé de todo, mañana, tarde y noche.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Desesperación tras el diagnóstico</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>EV20dccf8b1975</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Nombrar el diagnóstico + 'desesperación' + el probar-de-todo a ciegas resuena más que prometer un resultado estético.</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>El doctor me dijo: hay que operar, sacarte la vesícula. Algo dentro de mí dijo: tiene que haber otro camino.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Evitar el quirófano / vía natural</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>EV103445ddfd2a</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>El miedo a perder un órgano en cirugía es un disparador de entrada tan fuerte como el diagnóstico mismo.</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Me diagnosticaron hígado graso. Sin cirugía y sin pastillas de por vida, empecé a limpiarlo por lo natural.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Revertir natural / limpiar el hígado</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>EV395aeee91c7c</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>'Limpiarlo por lo natural, sin cirugía ni pastillas de por vida' convierte mejor que una promesa de síntoma.</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Hace un año me dieron hígado graso en grado preocupante. Hoy bajé 10 kilos y mi análisis salió limpio.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Prueba medible / revirtió lo irreversible</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>EV23ec746f6d9a</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>El testimonio de reversión con cifra (kilos + análisis limpio) supera a la promesa abstracta de 'sanar el hígado'.</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Un año siguiendo esto me hicieron ultrasonido y mi hígado salió limpio. Y no es mentira, revertí lo que decían irreversible.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Producto</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Prueba medible / ultrasonido limpio</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>EV551a30df75aa</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>El ultrasonido limpio como prueba de reversión de lo irreversible es el cierre más creíble para el público caliente MX.</t>
+        </is>
+      </c>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Cuando desperté con el diagnóstico, le entregué mi hígado a Dios y le pedí fuerza. Después busqué la herramienta natural correcta.</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Creyente / fe como marco</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Fe como marco / esperanza redentora</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>EVb25aac5fff83</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Un lead que honra la fe (entrega a Dios) sin prometer milagro conecta con el público caliente sin cruzar a la explotación.</t>
+        </is>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Le tenía miedo a lo natural: una amiga se intoxicó con moringa. ¿Y si esto choca con mi estatina?</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Objeción seguridad / interacción con medicina</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>EVa81d501174fa</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Nombrar de frente el miedo a intoxicarse y a la interacción con la estatina desarma la objeción #1 mejor que ignorarla.</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Me dijeron que el vinagre se contrapone con mi atorvastatina. Yo solo quería limpiar mi hígado sin hacerme daño.</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Objeción seguridad / interacción con medicina</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>EV4f66daea204a</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>El conflicto 'quiero lo natural pero choca con mi medicina' es el punto de dolor que abre a una dosis segura y probada.</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Nos diagnosticaron hígado graso, pero las mamás no tenemos tiempo de estar preparando el remedio todos los días.</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Villano DIY / facilidad de las gotas</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>EV6bf181681ddd</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>El dolor de 'no tener tiempo de preparar el remedio diario' posiciona las gotas como atajo mejor que un claim de eficacia.</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Núcleo Diagnóstico</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Después del diagnóstico probé el vinagre, el aceite con limón, los tés. Ayudaban a medias y era un martirio prepararlos.</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Villano DIY / remedios a medias</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>EVf1bed71ead4d</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Reconocer que los remedios caseros ayudan 'a medias' y cansan mantenerlos abre a 'lo mismo, concentrado y en la dosis correcta'.</t>
+        </is>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>¿El vinagre para el hígado choca con tu atorvastatina? Por eso lo natural también necesita la dosis correcta, no adivinar.</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>seguridad_interaccion_medicamento</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>EV4f66daea204a</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Nombrar la interacción estatina/remedio en el hook eleva CTR de la mujer medicada frente a un hook de beneficio genérico.</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Si ya tomas medicamento, esto no es para reemplazarlo: consúltalo con tu doctor. Lo natural, pero en la dosis correcta.</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>seguridad_consulta_medico</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>EVa975dbd810fc</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Un hook que admite límites ('no reemplaza tu medicina') genera más confianza y clics que uno que promete cura total.</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Una vecina tomó semillas de moringa por su cuenta y le hizo daño. Lo natural sin dosis correcta también lastima.</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Buscadora natural anti-sistema</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>seguridad_dosis_natural</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>EVa81d501174fa</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Anclar en un daño real por sobredosis natural valida la promesa 'dosis correcta' mejor que afirmarla en abstracto.</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>¿Los remedios para el hígado te irritan el intestino, te dan diarrea o dolor de panza? Estas gotas caen suaves, no te irritan.</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Intestino roto / colitis</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>seguridad_intestino_suave</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>EVecfdcb339361</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Prometer 'suave con tu intestino' (no 'seguro para tu hígado') convierte mejor al sub-avatar de colitis.</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Con gastritis, triglicéridos y colesterol altos, ¿qué es seguro tomar? Alcachofa y cardo mariano, en gotas, en la dosis justa.</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>seguridad_ingrediente_auditable</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>EVa7633fc26169</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Nombrar alcachofa y cardo mariano (ingredientes que ella audita) supera a un claim de 'fórmula natural' sin nombre.</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Ella siguió limpiando su hígado y el ultrasonido salió limpio. No fue milagro: fue constancia con la dosis correcta.</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Producto</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>prueba_ultrasonido_limpio</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>EV551a30df75aa</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>La prueba 'ultrasonido limpio' como resultado supera al claim de beneficio abstracto en el público caliente.</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Del 68% de grasa en el hígado bajó a 10% en dos meses. Cifra medible, no promesa: mídete antes y después.</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Producto</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>prueba_cifra_tiempo</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>EVec2e8ff832dc</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Una cifra concreta con tiempo ('68% a 10% en 2 meses') convierte mejor que un rango cualitativo tipo 'notarás mejoría'.</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Fue al ultrasonido y el médico se quedó sin palabras. Ella solo había limpiado su hígado, bien dosificado.</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Producto</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>prueba_ultrasonido_medico_sorprendido</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>EVfb3f73b5ebc0</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>El testimonio del 'médico sin palabras ante el ultrasonido' genera más credibilidad que un antes/después de peso.</t>
+        </is>
+      </c>
+      <c r="H24" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>La bilis digiere las grasas; si tu hígado va lento, viene la pesadez. Por eso la alcachofa ayuda: no es magia, es digestión.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Intestino roto / colitis</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>mecanismo_bilis_alcachofa</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>EVd6a1a1a6bb01</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Explicar el mecanismo bilis→pesadez con alcachofa (hecho respaldado) convierte mejor que 'desintoxica tu hígado' (palabra prohibida).</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Esa limpieza de hígado que intentas con remedios de la abuela, ahora concentrada, dosificada y en gotas. Sin adivinar cuántas hojas.</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Buscadora natural anti-sistema</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>mecanismo_limpiar_higado_dosificado</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>EV103445ddfd2a</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>El verbo nativo 'limpiar el hígado' + 'sin adivinar cuántas hojas' supera a lenguaje clínico o a 'detox'.</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>El aceite de oliva con limón en ayunas, todos los días, sanó hígados. ¿Y quién lo sostiene meses? Las gotas ya lo traen listo.</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Buscadora natural anti-sistema</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>villano_diy_ritual_diario</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>EV395aeee91c7c</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Atacar al villano DIY ('¿quién lo sostiene meses?') convierte mejor que atacar solo a la dieta o a las pastillas.</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Seguridad/Prueba</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Preparar el vinagre en cada comida, medir, no olvidar: por eso lo dejas. Las gotas hacen lo mismo, sin preparar nada diario.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Madre aterrada por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>villano_diy_preparar_diario</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>EV54ec0294eec2</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Describir el ritual exacto del vinagre y su fricción convierte mejor que un genérico 'sin complicaciones'.</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>POV: te das cuenta que no son gases… es grasa jajaja 😅 y ahí caí que era mi hígado.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Puente hinchazón→hígado como testimonio</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>EV9937651191c6</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>¿El avatar frío de TikTok acepta el salto de 'panza hinchada' a 'es mi hígado' cuando se enmarca como su propio chiste, no como claim médico?</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Ya no sé qué hacer, parezco embarazada 🥺 y no, no espero bebé: es mi panza inflada de siempre.</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Humillación social 'parezco embarazada'</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>EV896a667c600d</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>¿El dolor de entrada 'parezco embarazada' detiene el scroll del frío mejor que un ángulo de salud?</t>
+        </is>
+      </c>
+      <c r="H30" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Una señora me preguntó si estaba embarazada… y yo nomás con mi colitis 😔 me quería morir de vergüenza.</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Humillación social 'parezco embarazada'</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>EV9e5bfa9edeaa</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>¿La escena narrada del comentario ajeno genera más identificación que el enunciado abstracto de hinchazón?</t>
+        </is>
+      </c>
+      <c r="H31" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>En el camión dijeron que iban 2 embarazadas… era una embarazada y mi mamá con colitis nerviosa 😭😂</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Inconsciente</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Humillación social 'parezco embarazada'</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>EVb72cbfeeb711</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>¿Una historia de humillación en tercera persona (la mamá) desarma la defensa y aún así engancha por identificación?</t>
+        </is>
+      </c>
+      <c r="H32" s="24" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Esa panza de embarazada que traes… ni la regla tienes y ya andas hinchada 😂 no estás sola, amiga.</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Hinchazón constante no cíclica</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>EV772a697227e9</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>¿Nombrar que la panza está hinchada incluso fuera de la regla valida el problema como algo más que 'inflamación de mujer'?</t>
+        </is>
+      </c>
+      <c r="H33" s="24" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Mi panza ya está hinchada hasta cuando NO me baja 😂😂 dejé de creer que era normal.</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Hinchazón constante no cíclica</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>EV949d31514d28</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>¿El giro 'dejé de creer que era normal' mueve al avatar de resignación a búsqueda de solución dentro del mismo hook?</t>
+        </is>
+      </c>
+      <c r="H34" s="24" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>No estoy embarazada, tengo 8 meses de panza y cero bebé 🤣 y ya no la puedo meter aunque quiera.</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Inconsciente</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Humillación social 'parezco embarazada'</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>EV4d4015e6dbb4</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>¿La hipérbole cómica '8 meses de panza' funciona como hook de reconocimiento sin sonar burla del propio avatar?</t>
+        </is>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Yo viendo esto re hinchada, panzona, sin haber comido nada raro 😅 alguien más así o soy yo?</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Inconsciente</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Meta-reconocimiento en scroll</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>EV5d9200bf439f</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>¿El formato espejo ('tú, viendo esto, hinchada') genera comentarios de auto-identificación que alimentan alcance orgánico?</t>
+        </is>
+      </c>
+      <c r="H36" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Cualquier cosita que como me infla la barriga como globo 🎈 ya me da miedo sentarme a la mesa.</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Gatillo alimentario / miedo a comer</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>EV49bd7adae791</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>¿El ángulo 'ya me da miedo comer' abre la puerta al mecanismo digestión/bilis sin nombrar hígado todavía?</t>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Todo me cae mal, me siento inflamada y mi estómago es un huracán 😩 y todos me dicen que es normal.</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Problema</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Invalidación 'es normal'</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>EVef40d03a8002</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>¿Refutar el 'es normal' (bloating común pero no normal) posiciona la marca como la que sí la toma en serio?</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Llevo desde el 2021 con el estómago inflamado 🗣️ probé de todo y seguía pareciendo embarazada.</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Cronicidad / fatiga de soluciones</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>EV584c0fd179b4</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>¿La antigüedad del problema ('desde 2021') convierte curiosidad en intención porque ya agotó lo casero?</t>
+        </is>
+      </c>
+      <c r="H39" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Cabeza de Playa</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Muchas mujeres descubren que esa panza que odian no era gordura… era el hígado inflamado 🫢</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Consc. Solución</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>La hinchada humillada</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Puente hinchazón→hígado como testimonio</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>EVec2e8ff832dc</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>¿Presentar el puente panza→hígado en boca de 'muchas mujeres' (testimonio) pasa compliance y aún así intriga al frío?</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2393,7 +4190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2618,7 +4415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3288,7 +5085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3441,7 +5238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>